<commit_message>
fix: rebuild AIZ, AJG and AKAM DCFs on opus
The 2026-09-25 batch hit the weekly Fable limit and the orchestrator
re-spawned dcf-analyst on sonnet, below its tier. Re-judged on opus:
- AIZ: insurer FCFE at 9% CoE (OCF-capex counted premium float as owner
  cash); weighted IV 383.39 -> 339.51 vs 261.86
- AJG: debt was missing 1.52bn of credit-facility borrowings, basic not
  diluted shares, acquisition growth uncharged; 227.44 -> 247.01 vs 227.13
  (600m earnout payable is an estimate)
- AKAM: withholding taxes missing from SBC, SBC double-counted via
  post-SBC EBITDA, capitalized software missing from capex;
  22.28 -> 9.89 vs 110.41

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/research/AJG/Reports/AJG_DCF_Model.xlsx
+++ b/research/AJG/Reports/AJG_DCF_Model.xlsx
@@ -52,7 +52,7 @@
     <t xml:space="preserve">Price as of</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-24T20:00:03Z regular close (Yahoo Finance chart API); 52-week range 190.75-313.55</t>
+    <t xml:space="preserve">2026-09-24T20:00:03Z regular close (Yahoo Finance chart API)</t>
   </si>
   <si>
     <t xml:space="preserve">Balance sheet date</t>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Built at</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-25T09:32:59Z</t>
+    <t xml:space="preserve">2026-09-25T09:53:48Z</t>
   </si>
   <si>
     <t xml:space="preserve">Drivers file</t>
@@ -109,34 +109,34 @@
     <t xml:space="preserve">Methodology</t>
   </si>
   <si>
-    <t xml:space="preserve">summary: AJG is a capital-light, fee/commission-based global insurance brokerage (third/fourth-largest globally) with a decades-long algorithm of mid-single-digit organic growth plus continuous tuck-in M&amp;A, now digesting its largest-ever acquisition (AssuredPartners, $13.8B, closed August 2025). The valuation is built on an owner-FCF component DCF anchored to management's own (recently trimmed) FY2026 guidance rather than historical CAGRs, which are badly distorted by the AssuredPartners equity raise and deal-related D&amp;A/interest. Elevated D&amp;A (~7.5%-8% of revenue, mostly purchase-accounting intangible amortization) is genuinely non-cash and is added back correctly in the FCF build; the near-term normalized EBITDA margin (27.5% ramping to 30%) sits meaningfully below AJG's own guided Brokerage-segment-only EBITDAC range (33.6-34.2%) to reflect the lower-margin Risk Management mix and corporate costs, which is a deliberately conservative blend. FY2025 reported FCF ($1,785M, 12.8% margin) is a trough distorted by acquisition-close transaction costs and fiduciary-fund working-capital timing -- TTM OCF through Q2-2026 recovered to $2,449M -- so the base FCF for the DCF is built from normalized components rather than carried forward from the depressed FY2025 actual.
-key_risks_to_valuation: AssuredPartners integration execution -- the largest deal in company history; realizing $160M-$325M of targeted synergies carries meaningful execution risk, and management already removed an assumed Q4 2026 acceleration from guidance; Softening P&amp;C pricing cycle (property renewals -10% in Q2 2026) could spread into casualty/professional lines, which have so far remained firm and are propping up the organic growth guide; Elevated leverage (~3.0x net debt/EBITDA) narrows financial flexibility for further tuck-in M&amp;A and increases interest-expense sensitivity to rates; Premium valuation historically afforded to AJG (trailing P/E ~38-39x pre-cut) leaves little room for further guidance disappointments; Structural reliance on continuous, well-priced M&amp;A to sustain the growth algorithm; a thinner or more expensive acquisition pipeline would compress the long-run growth assumption; D&amp;A build is a modeling judgment (7.5% of revenue tapering to 6.0%) calibrated to disclosed intangible-amortization schedules but sensitive to the pace and size of future tuck-in acquisitions, which reset the amortization base each time</t>
+    <t xml:space="preserve">summary: AJG is valued as an asset-light fee business on an owner-FCF basis with ORGANIC growth only after FY2026; the tuck-in acquisition machine is treated as NPV-neutral rather than as free growth. Debt is the full 2026-06-30 combined debt including credit-facility borrowings; fiduciary cash is excluded; the remaining clean-energy tax credits and estimated earnout payables sit in the equity bridge.
+key_risks_to_valuation: Earnout payables are an estimate ($600M) -- each $260M is ~$1/share; Organic growth sensitivity to a prolonged soft P&amp;C pricing cycle; GAAP EBITDA margin path depends on AssuredPartners integration costs rolling off and $325M synergies landing; Excluding M&amp;A value understates AJG if its tuck-ins keep earning above WACC -- the main source of upside not in the model; Cash tax 24% on EBIT is a judgment; each 1pp is roughly $2/share</t>
   </si>
   <si>
     <t xml:space="preserve">Data sources</t>
   </si>
   <si>
     <t xml:space="preserve">price: Yahoo Finance chart API at inputs.price_as_of; 52-week range 190.75-313.55
-financials: research/AJG/Reports/AJG_Metrics.csv (core_metrics, SEC XBRL-sourced) plus direct SEC XBRL companyconcept API queries (CIK 0000354190) for FY2021-2025 capex (PaymentsForCapitalImprovements), D&amp;A (DepreciationAmortizationAndAccretionNet), SBC (ShareBasedCompensation), debt (LongTermDebtNoncurrent) and cash (CashCashEquivalentsRestrictedCashAndRestrictedCashEquivalents) to fill CapEx/FreeCashFlow gaps in the CSV for FY2023-2025, which the acquisition-era filings left unpopulated
-qualitative: research/AJG/Reports/AJG_Analysis.json (2026-09-25) -- AssuredPartners acquisition detail, September 2026 guidance cut, bull/bear cases, competitive position</t>
+financials: SEC XBRL companyfacts (CIK 0000354190): 10-K FY2025 and 10-Q Q2-2026 (period ended 2026-06-30) -- OCF, capex (PaymentsForCapitalImprovements), SBC, D&amp;A, interest expense, cash taxes paid, debt (DebtLongtermAndShorttermCombinedAmount), restricted cash, tax-credit DTA, intangible amortisation schedule, diluted EPS; research/AJG/Reports/AJG_Metrics.csv for history
+qualitative: research/AJG/Reports/AJG_Analysis.json (Sept-2026 investor update, Q2-2026 results, AP synergy targets)</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario narrative: bear</t>
   </si>
   <si>
-    <t xml:space="preserve">The September 2026 guidance cut is the leading edge of a broader P&amp;C pricing-cycle turn rather than a one-off Q4 timing fix; AssuredPartners integration underdelivers on its synergy targets as outsized brokerage mega-deals often do, elevated post-deal leverage constrains further tuck-in M&amp;A, and the mature margin stalls in the mid-to-high-20s% rather than reaching 30%+ -- though the recurring, high-retention commission base keeps growth modestly positive throughout rather than going negative.</t>
+    <t xml:space="preserve">The P&amp;C cycle turns fully soft for several years (property rates keep falling and casualty follows), contingent/supplemental commissions tied to carrier profitability compress, and AI-driven placement and embedded distribution erode small-commercial fees. Brokerage organic sinks to 2-3% (as in the 2015-17 soft market), AP integration slips and the synergies are reinvested to retain producers, so the margin stalls near 27%. Leverage (~3x) limits buybacks and the M&amp;A engine slows.</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario narrative: base</t>
   </si>
   <si>
-    <t xml:space="preserve">Management delivers its own just-lowered guidance (~5% Brokerage organic, 9-12% Risk Management organic) while AssuredPartners integration proceeds on the stated synergy timeline and AJG resumes its historical tuck-in M&amp;A pace; margin expands toward a ~30% mature adjusted EBITDA level via guided 40-60bps/yr underlying expansion plus synergy capture.</t>
+    <t xml:space="preserve">AJG meets its cut FY2026 guide (Brokerage organic ~5%, Gallagher Bassett 9-12%, ~6% blended) and then grows organically at 4-5% a year -- exposure-unit growth plus modest rate, with property renewal pricing (down ~10% in Q2-2026) weighing while casualty and professional lines stay firm. AssuredPartners integration runs on plan: $160M run-rate synergies by end-2026 and $325M by early 2028, and integration spend rolls off, lifting the GAAP EBITDA margin from ~26.5% to ~30% by Year 6. Tuck-in M&amp;A continues but is valued at zero NPV.</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario narrative: bull</t>
   </si>
   <si>
-    <t xml:space="preserve">AssuredPartners synergies beat the $325M ceiling and land early, Gallagher Bassett sustains the top of its double-digit organic range, casualty/professional-lines pricing strength offsets property softness so total organic growth reaccelerates, and disciplined tuck-in M&amp;A continues at historical pace -- pushing the mature margin toward the low-33% area.</t>
+    <t xml:space="preserve">The softening is confined to property and brief; casualty/social-inflation, cyber and benefits complexity keep advisory demand and premium inflation high, so Brokerage organic returns to 6-7% and Gallagher Bassett keeps compounding at double digits. AP synergies beat the $325M target and the shared-services centres keep adding 40-60bps a year, taking the margin to ~31.5% -- close to AJG's guided Brokerage adjusted EBITDAC once corporate costs are absorbed.</t>
   </si>
   <si>
     <t xml:space="preserve">Period</t>
@@ -532,7 +532,7 @@
     <t xml:space="preserve">Rate (%)</t>
   </si>
   <si>
-    <t xml:space="preserve">Value per share at 8.5% (WACC)</t>
+    <t xml:space="preserve">Value per share at 8% (WACC)</t>
   </si>
   <si>
     <t xml:space="preserve">Value per share at 9%</t>
@@ -2141,7 +2141,7 @@
         <v>85</v>
       </c>
       <c r="B3" s="3" t="n">
-        <v>256.3</v>
+        <v>259.3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2149,7 +2149,7 @@
         <v>86</v>
       </c>
       <c r="B4" s="3" t="n">
-        <v>10569</v>
+        <v>12472</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2157,7 +2157,7 @@
         <v>87</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0</v>
+        <v>-100</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2240,7 +2240,7 @@
         <v>105</v>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3</v>
+        <v>18.5</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>2.5</v>
@@ -2249,25 +2249,25 @@
         <v>3</v>
       </c>
       <c r="F13" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="I13" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="3" t="n">
+      <c r="J13" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="K13" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="L13" s="3" t="n">
         <v>2.5</v>
-      </c>
-      <c r="J13" s="3" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="K13" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2275,22 +2275,22 @@
         <v>106</v>
       </c>
       <c r="C14" s="3" t="n">
-        <v>25.5</v>
+        <v>26</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>25.5</v>
+        <v>26.5</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>27</v>
@@ -2310,34 +2310,34 @@
         <v>107</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="G15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="J15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2380,34 +2380,34 @@
         <v>109</v>
       </c>
       <c r="C17" s="3" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>7.8</v>
+        <v>7.5</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>7.6</v>
+        <v>7</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>7.6</v>
+        <v>6.5</v>
       </c>
       <c r="G17" s="3" t="n">
-        <v>7.4</v>
+        <v>6</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>7.4</v>
+        <v>5</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>7.2</v>
+        <v>4</v>
       </c>
       <c r="J17" s="3" t="n">
-        <v>7.2</v>
+        <v>3</v>
       </c>
       <c r="K17" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L17" s="3" t="n">
-        <v>7</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2415,34 +2415,34 @@
         <v>110</v>
       </c>
       <c r="C18" s="3" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>1.3</v>
+        <v>1.1</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>1.25</v>
+        <v>1.1</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>1.25</v>
+        <v>1.1</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2450,34 +2450,34 @@
         <v>111</v>
       </c>
       <c r="C19" s="3" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2485,7 +2485,7 @@
         <v>112</v>
       </c>
       <c r="B20" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2493,7 +2493,7 @@
         <v>113</v>
       </c>
       <c r="B21" s="3" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2501,7 +2501,7 @@
         <v>114</v>
       </c>
       <c r="B22" s="3" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2517,7 +2517,7 @@
         <v>116</v>
       </c>
       <c r="B24" s="3" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2560,34 +2560,34 @@
         <v>105</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>7.5</v>
+        <v>19.4</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="F27" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="J27" s="3" t="n">
         <v>4</v>
       </c>
       <c r="K27" s="3" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2595,10 +2595,10 @@
         <v>106</v>
       </c>
       <c r="C28" s="3" t="n">
+        <v>26.5</v>
+      </c>
+      <c r="D28" s="3" t="n">
         <v>27.5</v>
-      </c>
-      <c r="D28" s="3" t="n">
-        <v>28</v>
       </c>
       <c r="E28" s="3" t="n">
         <v>28.5</v>
@@ -2630,34 +2630,34 @@
         <v>107</v>
       </c>
       <c r="C29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="F29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="J29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="K29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2700,34 +2700,34 @@
         <v>109</v>
       </c>
       <c r="C31" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="D31" s="3" t="n">
         <v>7.5</v>
       </c>
-      <c r="D31" s="3" t="n">
-        <v>7.3</v>
-      </c>
       <c r="E31" s="3" t="n">
-        <v>7.1</v>
+        <v>7</v>
       </c>
       <c r="F31" s="3" t="n">
-        <v>6.9</v>
+        <v>6.5</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>6.7</v>
+        <v>6</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>6.3</v>
+        <v>4</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>6.2</v>
+        <v>3</v>
       </c>
       <c r="K31" s="3" t="n">
-        <v>6.1</v>
+        <v>2</v>
       </c>
       <c r="L31" s="3" t="n">
-        <v>6</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2735,10 +2735,10 @@
         <v>110</v>
       </c>
       <c r="C32" s="3" t="n">
-        <v>1.2</v>
+        <v>1.1</v>
       </c>
       <c r="D32" s="3" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="E32" s="3" t="n">
         <v>1.1</v>
@@ -2747,22 +2747,22 @@
         <v>1.1</v>
       </c>
       <c r="G32" s="3" t="n">
-        <v>1.05</v>
+        <v>1.1</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>1.05</v>
+        <v>1.1</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="J32" s="3" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="K32" s="3" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="L32" s="3" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2770,34 +2770,34 @@
         <v>111</v>
       </c>
       <c r="C33" s="3" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D33" s="3" t="n">
-        <v>19.5</v>
+        <v>24</v>
       </c>
       <c r="E33" s="3" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F33" s="3" t="n">
-        <v>20.5</v>
+        <v>24</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="L33" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2805,7 +2805,7 @@
         <v>112</v>
       </c>
       <c r="B34" s="3" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2813,7 +2813,7 @@
         <v>113</v>
       </c>
       <c r="B35" s="3" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2821,7 +2821,7 @@
         <v>114</v>
       </c>
       <c r="B36" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2837,7 +2837,7 @@
         <v>116</v>
       </c>
       <c r="B38" s="3" t="n">
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2880,34 +2880,34 @@
         <v>105</v>
       </c>
       <c r="C41" s="3" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D41" s="3" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E41" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F41" s="3" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="G41" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="K41" s="3" t="n">
         <v>4</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2915,34 +2915,34 @@
         <v>106</v>
       </c>
       <c r="C42" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="D42" s="3" t="n">
         <v>28.5</v>
       </c>
-      <c r="D42" s="3" t="n">
+      <c r="E42" s="3" t="n">
         <v>29.5</v>
       </c>
-      <c r="E42" s="3" t="n">
+      <c r="F42" s="3" t="n">
         <v>30.5</v>
       </c>
-      <c r="F42" s="3" t="n">
+      <c r="G42" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="H42" s="3" t="n">
         <v>31.5</v>
       </c>
-      <c r="G42" s="3" t="n">
-        <v>32</v>
-      </c>
-      <c r="H42" s="3" t="n">
-        <v>32.5</v>
-      </c>
       <c r="I42" s="3" t="n">
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="J42" s="3" t="n">
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="K42" s="3" t="n">
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="L42" s="3" t="n">
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2950,34 +2950,34 @@
         <v>107</v>
       </c>
       <c r="C43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="D43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="E43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="F43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="G43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="J43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="L43" s="3" t="n">
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3020,34 +3020,34 @@
         <v>109</v>
       </c>
       <c r="C45" s="3" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
       <c r="D45" s="3" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="E45" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="E45" s="3" t="n">
-        <v>6.7</v>
-      </c>
       <c r="F45" s="3" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="G45" s="3" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>5.9</v>
+        <v>5</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>5.7</v>
+        <v>4</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>5.4</v>
+        <v>2</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>5.3</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3055,34 +3055,34 @@
         <v>110</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>1.15</v>
+        <v>1.1</v>
       </c>
       <c r="D46" s="3" t="n">
         <v>1.1</v>
       </c>
       <c r="E46" s="3" t="n">
-        <v>1.05</v>
+        <v>1.1</v>
       </c>
       <c r="F46" s="3" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="G46" s="3" t="n">
-        <v>1</v>
+        <v>1.1</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>0.95</v>
+        <v>1.1</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>0.95</v>
+        <v>1.1</v>
       </c>
       <c r="J46" s="3" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="K46" s="3" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
       <c r="L46" s="3" t="n">
-        <v>0.9</v>
+        <v>1.1</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3090,34 +3090,34 @@
         <v>111</v>
       </c>
       <c r="C47" s="3" t="n">
-        <v>18.5</v>
+        <v>24</v>
       </c>
       <c r="D47" s="3" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E47" s="3" t="n">
-        <v>19.5</v>
+        <v>24</v>
       </c>
       <c r="F47" s="3" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G47" s="3" t="n">
-        <v>20.5</v>
+        <v>24</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J47" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K47" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="L47" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3279,7 +3279,7 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C13</f>
-        <v>3</v>
+        <v>18.5</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">Assumptions!D13</f>
@@ -3291,31 +3291,31 @@
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">Assumptions!F13</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="G5" s="4" t="n">
         <f aca="false">Assumptions!G13</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="H5" s="4" t="n">
         <f aca="false">Assumptions!H13</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="I5" s="4" t="n">
         <f aca="false">Assumptions!I13</f>
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="J5" s="4" t="n">
         <f aca="false">Assumptions!J13</f>
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="K5" s="4" t="n">
         <f aca="false">Assumptions!K13</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L5" s="4" t="n">
         <f aca="false">Assumptions!L13</f>
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3327,43 +3327,43 @@
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">B6*(1+C5/100)</f>
-        <v>14360.26</v>
+        <v>16521.27</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">C6*(1+D5/100)</f>
-        <v>14719.2665</v>
+        <v>16934.30175</v>
       </c>
       <c r="E6" s="0" t="n">
         <f aca="false">D6*(1+E5/100)</f>
-        <v>15160.844495</v>
+        <v>17442.3308025</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">E6*(1+F5/100)</f>
-        <v>15615.66982985</v>
+        <v>18052.8123805875</v>
       </c>
       <c r="G6" s="0" t="n">
         <f aca="false">F6*(1+G5/100)</f>
-        <v>16084.1399247455</v>
+        <v>18684.6608139081</v>
       </c>
       <c r="H6" s="0" t="n">
         <f aca="false">G6*(1+H5/100)</f>
-        <v>16566.6641224879</v>
+        <v>19338.6239423948</v>
       </c>
       <c r="I6" s="0" t="n">
         <f aca="false">H6*(1+I5/100)</f>
-        <v>16980.8307255501</v>
+        <v>19918.7826606667</v>
       </c>
       <c r="J6" s="0" t="n">
         <f aca="false">I6*(1+J5/100)</f>
-        <v>17405.3514936888</v>
+        <v>20516.3461404867</v>
       </c>
       <c r="K6" s="0" t="n">
         <f aca="false">J6*(1+K5/100)</f>
-        <v>17753.4585235626</v>
+        <v>21131.8365247013</v>
       </c>
       <c r="L6" s="0" t="n">
         <f aca="false">K6*(1+L5/100)</f>
-        <v>18108.5276940338</v>
+        <v>21660.1324378188</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3372,27 +3372,27 @@
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C14</f>
-        <v>25.5</v>
+        <v>26</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">Assumptions!D14</f>
-        <v>25.5</v>
+        <v>26.5</v>
       </c>
       <c r="E7" s="4" t="n">
         <f aca="false">Assumptions!E14</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="F7" s="4" t="n">
         <f aca="false">Assumptions!F14</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="G7" s="4" t="n">
         <f aca="false">Assumptions!G14</f>
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="H7" s="4" t="n">
         <f aca="false">Assumptions!H14</f>
-        <v>26.5</v>
+        <v>27</v>
       </c>
       <c r="I7" s="4" t="n">
         <f aca="false">Assumptions!I14</f>
@@ -3417,43 +3417,43 @@
       </c>
       <c r="C8" s="0" t="n">
         <f aca="false">C6*C7/100</f>
-        <v>3661.8663</v>
+        <v>4295.5302</v>
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">D6*D7/100</f>
-        <v>3753.4129575</v>
+        <v>4487.58996375</v>
       </c>
       <c r="E8" s="0" t="n">
         <f aca="false">E6*E7/100</f>
-        <v>3941.8195687</v>
+        <v>4709.429316675</v>
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">F6*F7/100</f>
-        <v>4060.074155761</v>
+        <v>4874.25934275863</v>
       </c>
       <c r="G8" s="0" t="n">
         <f aca="false">G6*G7/100</f>
-        <v>4262.29708005756</v>
+        <v>5044.85841975518</v>
       </c>
       <c r="H8" s="0" t="n">
         <f aca="false">H6*H7/100</f>
-        <v>4390.16599245929</v>
+        <v>5221.42846444661</v>
       </c>
       <c r="I8" s="0" t="n">
         <f aca="false">I6*I7/100</f>
-        <v>4584.82429589852</v>
+        <v>5378.07131838001</v>
       </c>
       <c r="J8" s="0" t="n">
         <f aca="false">J6*J7/100</f>
-        <v>4699.44490329598</v>
+        <v>5539.41345793141</v>
       </c>
       <c r="K8" s="0" t="n">
         <f aca="false">K6*K7/100</f>
-        <v>4793.4338013619</v>
+        <v>5705.59586166935</v>
       </c>
       <c r="L8" s="0" t="n">
         <f aca="false">L6*L7/100</f>
-        <v>4889.30247738914</v>
+        <v>5848.23575821108</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3462,43 +3462,43 @@
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Assumptions!D15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">Assumptions!E15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">Assumptions!F15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="G9" s="4" t="n">
         <f aca="false">Assumptions!G15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">Assumptions!H15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="I9" s="4" t="n">
         <f aca="false">Assumptions!I15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="J9" s="4" t="n">
         <f aca="false">Assumptions!J15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="K9" s="4" t="n">
         <f aca="false">Assumptions!K15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
       <c r="L9" s="4" t="n">
         <f aca="false">Assumptions!L15</f>
-        <v>0.35</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3507,43 +3507,43 @@
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
-        <v>-50.26091</v>
+        <v>-82.60635</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">-D6*D9/100</f>
-        <v>-51.51743275</v>
+        <v>-84.67150875</v>
       </c>
       <c r="E10" s="0" t="n">
         <f aca="false">-E6*E9/100</f>
-        <v>-53.0629557325</v>
+        <v>-87.2116540125</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">-F6*F9/100</f>
-        <v>-54.654844404475</v>
+        <v>-90.2640619029375</v>
       </c>
       <c r="G10" s="0" t="n">
         <f aca="false">-G6*G9/100</f>
-        <v>-56.2944897366093</v>
+        <v>-93.4233040695403</v>
       </c>
       <c r="H10" s="0" t="n">
         <f aca="false">-H6*H9/100</f>
-        <v>-57.9833244287075</v>
+        <v>-96.6931197119742</v>
       </c>
       <c r="I10" s="0" t="n">
         <f aca="false">-I6*I9/100</f>
-        <v>-59.4329075394252</v>
+        <v>-99.5939133033334</v>
       </c>
       <c r="J10" s="0" t="n">
         <f aca="false">-J6*J9/100</f>
-        <v>-60.9187302279109</v>
+        <v>-102.581730702433</v>
       </c>
       <c r="K10" s="0" t="n">
         <f aca="false">-K6*K9/100</f>
-        <v>-62.1371048324691</v>
+        <v>-105.659182623506</v>
       </c>
       <c r="L10" s="0" t="n">
         <f aca="false">-L6*L9/100</f>
-        <v>-63.3798469291184</v>
+        <v>-108.300662189094</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3552,43 +3552,43 @@
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
-        <v>3611.60539</v>
+        <v>4212.92385</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">D8+D10+D24</f>
-        <v>3701.89552475</v>
+        <v>4402.918455</v>
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">E8+E10+E24</f>
-        <v>3888.7566129675</v>
+        <v>4622.2176626625</v>
       </c>
       <c r="F11" s="0" t="n">
         <f aca="false">F8+F10+F24</f>
-        <v>4005.41931135652</v>
+        <v>4783.99528085569</v>
       </c>
       <c r="G11" s="0" t="n">
         <f aca="false">G8+G10+G24</f>
-        <v>4206.00259032095</v>
+        <v>4951.43511568564</v>
       </c>
       <c r="H11" s="0" t="n">
         <f aca="false">H8+H10+H24</f>
-        <v>4332.18266803058</v>
+        <v>5124.73534473463</v>
       </c>
       <c r="I11" s="0" t="n">
         <f aca="false">I8+I10+I24</f>
-        <v>4525.39138835909</v>
+        <v>5278.47740507667</v>
       </c>
       <c r="J11" s="0" t="n">
         <f aca="false">J8+J10+J24</f>
-        <v>4638.52617306807</v>
+        <v>5436.83172722897</v>
       </c>
       <c r="K11" s="0" t="n">
         <f aca="false">K8+K10+K24</f>
-        <v>4731.29669652943</v>
+        <v>5599.93667904584</v>
       </c>
       <c r="L11" s="0" t="n">
         <f aca="false">L8+L10+L24</f>
-        <v>4825.92263046002</v>
+        <v>5739.93509602199</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3597,43 +3597,43 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C17/100</f>
-        <v>-1120.10028</v>
+        <v>-1321.7016</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">-D6*Assumptions!D17/100</f>
-        <v>-1148.102787</v>
+        <v>-1270.07263125</v>
       </c>
       <c r="E12" s="4" t="n">
         <f aca="false">-E6*Assumptions!E17/100</f>
-        <v>-1152.22418162</v>
+        <v>-1220.963156175</v>
       </c>
       <c r="F12" s="4" t="n">
         <f aca="false">-F6*Assumptions!F17/100</f>
-        <v>-1186.7909070686</v>
+        <v>-1173.43280473819</v>
       </c>
       <c r="G12" s="4" t="n">
         <f aca="false">-G6*Assumptions!G17/100</f>
-        <v>-1190.22635443117</v>
+        <v>-1121.07964883448</v>
       </c>
       <c r="H12" s="4" t="n">
         <f aca="false">-H6*Assumptions!H17/100</f>
-        <v>-1225.9331450641</v>
+        <v>-966.931197119742</v>
       </c>
       <c r="I12" s="4" t="n">
         <f aca="false">-I6*Assumptions!I17/100</f>
-        <v>-1222.6198122396</v>
+        <v>-796.751306426667</v>
       </c>
       <c r="J12" s="4" t="n">
         <f aca="false">-J6*Assumptions!J17/100</f>
-        <v>-1253.18530754559</v>
+        <v>-615.490384214601</v>
       </c>
       <c r="K12" s="4" t="n">
         <f aca="false">-K6*Assumptions!K17/100</f>
-        <v>-1242.74209664938</v>
+        <v>-422.636730494026</v>
       </c>
       <c r="L12" s="4" t="n">
         <f aca="false">-L6*Assumptions!L17/100</f>
-        <v>-1267.59693858237</v>
+        <v>-238.261456816007</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3642,43 +3642,43 @@
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
-        <v>2491.50511</v>
+        <v>2891.22225</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">D11+D12</f>
-        <v>2553.79273775</v>
+        <v>3132.84582375</v>
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">E11+E12</f>
-        <v>2736.5324313475</v>
+        <v>3401.2545064875</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">F11+F12</f>
-        <v>2818.62840428793</v>
+        <v>3610.5624761175</v>
       </c>
       <c r="G13" s="0" t="n">
         <f aca="false">G11+G12</f>
-        <v>3015.77623588978</v>
+        <v>3830.35546685115</v>
       </c>
       <c r="H13" s="0" t="n">
         <f aca="false">H11+H12</f>
-        <v>3106.24952296648</v>
+        <v>4157.80414761489</v>
       </c>
       <c r="I13" s="0" t="n">
         <f aca="false">I11+I12</f>
-        <v>3302.77157611949</v>
+        <v>4481.72609865</v>
       </c>
       <c r="J13" s="0" t="n">
         <f aca="false">J11+J12</f>
-        <v>3385.34086552247</v>
+        <v>4821.34134301437</v>
       </c>
       <c r="K13" s="0" t="n">
         <f aca="false">K11+K12</f>
-        <v>3488.55459988005</v>
+        <v>5177.29994855182</v>
       </c>
       <c r="L13" s="0" t="n">
         <f aca="false">L11+L12</f>
-        <v>3558.32569187765</v>
+        <v>5501.67363920598</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3687,43 +3687,43 @@
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C19</f>
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D14" s="4" t="n">
         <f aca="false">Assumptions!D19</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E14" s="4" t="n">
         <f aca="false">Assumptions!E19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F14" s="4" t="n">
         <f aca="false">Assumptions!F19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="G14" s="4" t="n">
         <f aca="false">Assumptions!G19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H14" s="4" t="n">
         <f aca="false">Assumptions!H19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="I14" s="4" t="n">
         <f aca="false">Assumptions!I19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="J14" s="4" t="n">
         <f aca="false">Assumptions!J19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="K14" s="4" t="n">
         <f aca="false">Assumptions!K19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="L14" s="4" t="n">
         <f aca="false">Assumptions!L19</f>
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3732,43 +3732,43 @@
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
-        <v>1993.204088</v>
+        <v>2197.32891</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">D13-MAX(0,D13)*D14/100</f>
-        <v>2017.4962628225</v>
+        <v>2380.96282605</v>
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">E13-MAX(0,E13)*E14/100</f>
-        <v>2134.49529645105</v>
+        <v>2584.9534249305</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">F13-MAX(0,F13)*F14/100</f>
-        <v>2198.53015534458</v>
+        <v>2744.0274818493</v>
       </c>
       <c r="G15" s="0" t="n">
         <f aca="false">G13-MAX(0,G13)*G14/100</f>
-        <v>2352.30546399403</v>
+        <v>2911.07015480688</v>
       </c>
       <c r="H15" s="0" t="n">
         <f aca="false">H13-MAX(0,H13)*H14/100</f>
-        <v>2422.87462791385</v>
+        <v>3159.93115218732</v>
       </c>
       <c r="I15" s="0" t="n">
         <f aca="false">I13-MAX(0,I13)*I14/100</f>
-        <v>2576.1618293732</v>
+        <v>3406.111834974</v>
       </c>
       <c r="J15" s="0" t="n">
         <f aca="false">J13-MAX(0,J13)*J14/100</f>
-        <v>2640.56587510753</v>
+        <v>3664.21942069092</v>
       </c>
       <c r="K15" s="0" t="n">
         <f aca="false">K13-MAX(0,K13)*K14/100</f>
-        <v>2721.07258790644</v>
+        <v>3934.74796089938</v>
       </c>
       <c r="L15" s="0" t="n">
         <f aca="false">L13-MAX(0,L13)*L14/100</f>
-        <v>2775.49403966457</v>
+        <v>4181.27196579654</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3777,43 +3777,43 @@
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
-        <v>1120.10028</v>
+        <v>1321.7016</v>
       </c>
       <c r="D16" s="0" t="n">
         <f aca="false">-D12</f>
-        <v>1148.102787</v>
+        <v>1270.07263125</v>
       </c>
       <c r="E16" s="0" t="n">
         <f aca="false">-E12</f>
-        <v>1152.22418162</v>
+        <v>1220.963156175</v>
       </c>
       <c r="F16" s="0" t="n">
         <f aca="false">-F12</f>
-        <v>1186.7909070686</v>
+        <v>1173.43280473819</v>
       </c>
       <c r="G16" s="0" t="n">
         <f aca="false">-G12</f>
-        <v>1190.22635443117</v>
+        <v>1121.07964883448</v>
       </c>
       <c r="H16" s="0" t="n">
         <f aca="false">-H12</f>
-        <v>1225.9331450641</v>
+        <v>966.931197119742</v>
       </c>
       <c r="I16" s="0" t="n">
         <f aca="false">-I12</f>
-        <v>1222.6198122396</v>
+        <v>796.751306426667</v>
       </c>
       <c r="J16" s="0" t="n">
         <f aca="false">-J12</f>
-        <v>1253.18530754559</v>
+        <v>615.490384214601</v>
       </c>
       <c r="K16" s="0" t="n">
         <f aca="false">-K12</f>
-        <v>1242.74209664938</v>
+        <v>422.636730494026</v>
       </c>
       <c r="L16" s="0" t="n">
         <f aca="false">-L12</f>
-        <v>1267.59693858237</v>
+        <v>238.261456816007</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3822,43 +3822,43 @@
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C18/100</f>
-        <v>-186.68338</v>
+        <v>-181.73397</v>
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">-D6*Assumptions!D18/100</f>
-        <v>-191.3504645</v>
+        <v>-186.27731925</v>
       </c>
       <c r="E17" s="4" t="n">
         <f aca="false">-E6*Assumptions!E18/100</f>
-        <v>-189.5105561875</v>
+        <v>-191.8656388275</v>
       </c>
       <c r="F17" s="4" t="n">
         <f aca="false">-F6*Assumptions!F18/100</f>
-        <v>-195.195872873125</v>
+        <v>-198.580936186463</v>
       </c>
       <c r="G17" s="4" t="n">
         <f aca="false">-G6*Assumptions!G18/100</f>
-        <v>-193.009679096946</v>
+        <v>-205.531268952989</v>
       </c>
       <c r="H17" s="4" t="n">
         <f aca="false">-H6*Assumptions!H18/100</f>
-        <v>-198.799969469854</v>
+        <v>-212.724863366343</v>
       </c>
       <c r="I17" s="4" t="n">
         <f aca="false">-I6*Assumptions!I18/100</f>
-        <v>-203.769968706601</v>
+        <v>-219.106609267334</v>
       </c>
       <c r="J17" s="4" t="n">
         <f aca="false">-J6*Assumptions!J18/100</f>
-        <v>-208.864217924266</v>
+        <v>-225.679807545354</v>
       </c>
       <c r="K17" s="4" t="n">
         <f aca="false">-K6*Assumptions!K18/100</f>
-        <v>-213.041502282751</v>
+        <v>-232.450201771714</v>
       </c>
       <c r="L17" s="4" t="n">
         <f aca="false">-L6*Assumptions!L18/100</f>
-        <v>-217.302332328406</v>
+        <v>-238.261456816007</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3912,43 +3912,43 @@
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
-        <v>2926.620988</v>
+        <v>3337.29654</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">D15+D16+D17+D18</f>
-        <v>2974.2485853225</v>
+        <v>3464.75813805</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">E15+E16+E17+E18</f>
-        <v>3097.20892188355</v>
+        <v>3614.050942278</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">F15+F16+F17+F18</f>
-        <v>3190.12518954006</v>
+        <v>3718.87935040103</v>
       </c>
       <c r="G19" s="0" t="n">
         <f aca="false">G15+G16+G17+G18</f>
-        <v>3349.52213932825</v>
+        <v>3826.61853468837</v>
       </c>
       <c r="H19" s="0" t="n">
         <f aca="false">H15+H16+H17+H18</f>
-        <v>3450.0078035081</v>
+        <v>3914.13748594072</v>
       </c>
       <c r="I19" s="0" t="n">
         <f aca="false">I15+I16+I17+I18</f>
-        <v>3595.0116729062</v>
+        <v>3983.75653213334</v>
       </c>
       <c r="J19" s="0" t="n">
         <f aca="false">J15+J16+J17+J18</f>
-        <v>3684.88696472886</v>
+        <v>4054.02999736017</v>
       </c>
       <c r="K19" s="0" t="n">
         <f aca="false">K15+K16+K17+K18</f>
-        <v>3750.77318227307</v>
+        <v>4124.93448962169</v>
       </c>
       <c r="L19" s="0" t="n">
         <f aca="false">L15+L16+L17+L18</f>
-        <v>3825.78864591853</v>
+        <v>4181.27196579654</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3957,43 +3957,43 @@
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
-        <v>0.909090909090909</v>
+        <v>0.925925925925926</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^D4</f>
-        <v>0.826446280991735</v>
+        <v>0.857338820301783</v>
       </c>
       <c r="E20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^E4</f>
-        <v>0.751314800901578</v>
+        <v>0.79383224102017</v>
       </c>
       <c r="F20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^F4</f>
-        <v>0.683013455365071</v>
+        <v>0.735029852796453</v>
       </c>
       <c r="G20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^G4</f>
-        <v>0.620921323059155</v>
+        <v>0.680583197033753</v>
       </c>
       <c r="H20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^H4</f>
-        <v>0.564473930053777</v>
+        <v>0.630169626883105</v>
       </c>
       <c r="I20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^I4</f>
-        <v>0.513158118230707</v>
+        <v>0.583490395262134</v>
       </c>
       <c r="J20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^J4</f>
-        <v>0.466507380209733</v>
+        <v>0.540268884501976</v>
       </c>
       <c r="K20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^K4</f>
-        <v>0.424097618372485</v>
+        <v>0.500248967131459</v>
       </c>
       <c r="L20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^L4</f>
-        <v>0.385543289429531</v>
+        <v>0.463193488084684</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4002,43 +4002,43 @@
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
-        <v>2660.56453454545</v>
+        <v>3090.08938888889</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">D19*D20</f>
-        <v>2458.05668208471</v>
+        <v>2970.47165470679</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">E19*E20</f>
-        <v>2326.97890449553</v>
+        <v>2868.9501586696</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">F19*F20</f>
-        <v>2178.8984287549</v>
+        <v>2733.48734149304</v>
       </c>
       <c r="G21" s="0" t="n">
         <f aca="false">G19*G20</f>
-        <v>2079.78971836763</v>
+        <v>2604.33227616683</v>
       </c>
       <c r="H21" s="0" t="n">
         <f aca="false">H19*H20</f>
-        <v>1947.43946356242</v>
+        <v>2466.57055908443</v>
       </c>
       <c r="I21" s="0" t="n">
         <f aca="false">I19*I20</f>
-        <v>1844.80942508597</v>
+        <v>2324.48367356259</v>
       </c>
       <c r="J21" s="0" t="n">
         <f aca="false">J19*J20</f>
-        <v>1719.02696428466</v>
+        <v>2190.26626441133</v>
       </c>
       <c r="K21" s="0" t="n">
         <f aca="false">K19*K20</f>
-        <v>1590.69397365739</v>
+        <v>2063.49421791818</v>
       </c>
       <c r="L21" s="0" t="n">
         <f aca="false">L19*L20</f>
-        <v>1475.00713920958</v>
+        <v>1936.73794646801</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4142,7 +4142,7 @@
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$20</f>
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$21</f>
-        <v>2</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4160,7 +4160,7 @@
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$22</f>
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4169,7 +4169,7 @@
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
-        <v>20281.2652340482</v>
+        <v>25248.8834813697</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
-        <v>3825.78864591853</v>
+        <v>4181.27196579654</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4187,7 +4187,7 @@
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
-        <v>48778.8052354612</v>
+        <v>77923.7048171174</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4196,7 +4196,7 @@
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
-        <v>53561.0410428594</v>
+        <v>66900.3514527447</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
-        <v>48778.8052354612</v>
+        <v>66900.3514527447</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
-        <v>18806.3410249222</v>
+        <v>30987.8071434881</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4223,7 +4223,7 @@
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
-        <v>39087.6062589704</v>
+        <v>56236.6906248578</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
-        <v>28518.6062589704</v>
+        <v>43664.6906248578</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4241,7 +4241,7 @@
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>111.27041068658</v>
+        <v>168.39448756212</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4250,7 +4250,7 @@
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>-0.510102537372519</v>
+        <v>-0.258598654681811</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4259,7 +4259,7 @@
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
-        <v>342.855018361561</v>
+        <v>625.727001061877</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
-        <v>311.554852024554</v>
+        <v>934.877554877795</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4277,7 +4277,7 @@
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>113.823707098543</v>
+        <v>174.413016509053</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
-        <v>30017.7262987454</v>
+        <v>34286.4301195317</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4304,7 +4304,7 @@
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>51.6192428477828</v>
+        <v>56.1173485238053</v>
       </c>
     </row>
   </sheetData>
@@ -4426,31 +4426,31 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C27</f>
-        <v>7.5</v>
+        <v>19.4</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">Assumptions!D27</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">Assumptions!E27</f>
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">Assumptions!F27</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G5" s="4" t="n">
         <f aca="false">Assumptions!G27</f>
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="H5" s="4" t="n">
         <f aca="false">Assumptions!H27</f>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="I5" s="4" t="n">
         <f aca="false">Assumptions!I27</f>
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="J5" s="4" t="n">
         <f aca="false">Assumptions!J27</f>
@@ -4458,11 +4458,11 @@
       </c>
       <c r="K5" s="4" t="n">
         <f aca="false">Assumptions!K27</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="L5" s="4" t="n">
         <f aca="false">Assumptions!L27</f>
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4474,43 +4474,43 @@
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">B6*(1+C5/100)</f>
-        <v>14987.65</v>
+        <v>16646.748</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">C6*(1+D5/100)</f>
-        <v>16036.7855</v>
+        <v>17479.0854</v>
       </c>
       <c r="E6" s="0" t="n">
         <f aca="false">D6*(1+E5/100)</f>
-        <v>17079.1765575</v>
+        <v>18353.03967</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">E6*(1+F5/100)</f>
-        <v>18103.92715095</v>
+        <v>19270.6916535</v>
       </c>
       <c r="G6" s="0" t="n">
         <f aca="false">F6*(1+G5/100)</f>
-        <v>19099.6431442522</v>
+        <v>20137.8727779075</v>
       </c>
       <c r="H6" s="0" t="n">
         <f aca="false">G6*(1+H5/100)</f>
-        <v>20054.6253014649</v>
+        <v>21044.0770529133</v>
       </c>
       <c r="I6" s="0" t="n">
         <f aca="false">H6*(1+I5/100)</f>
-        <v>20957.0834400308</v>
+        <v>21885.8401350299</v>
       </c>
       <c r="J6" s="0" t="n">
         <f aca="false">I6*(1+J5/100)</f>
-        <v>21795.366777632</v>
+        <v>22761.2737404311</v>
       </c>
       <c r="K6" s="0" t="n">
         <f aca="false">J6*(1+K5/100)</f>
-        <v>22449.227780961</v>
+        <v>23557.9183213462</v>
       </c>
       <c r="L6" s="0" t="n">
         <f aca="false">K6*(1+L5/100)</f>
-        <v>23010.458475485</v>
+        <v>24382.4454625933</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4519,11 +4519,11 @@
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C28</f>
-        <v>27.5</v>
+        <v>26.5</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">Assumptions!D28</f>
-        <v>28</v>
+        <v>27.5</v>
       </c>
       <c r="E7" s="4" t="n">
         <f aca="false">Assumptions!E28</f>
@@ -4564,43 +4564,43 @@
       </c>
       <c r="C8" s="0" t="n">
         <f aca="false">C6*C7/100</f>
-        <v>4121.60375</v>
+        <v>4411.38822</v>
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">D6*D7/100</f>
-        <v>4490.29994</v>
+        <v>4806.748485</v>
       </c>
       <c r="E8" s="0" t="n">
         <f aca="false">E6*E7/100</f>
-        <v>4867.5653188875</v>
+        <v>5230.61630595</v>
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">F6*F7/100</f>
-        <v>5250.1388737755</v>
+        <v>5588.500579515</v>
       </c>
       <c r="G8" s="0" t="n">
         <f aca="false">G6*G7/100</f>
-        <v>5634.39472755441</v>
+        <v>5940.67246948271</v>
       </c>
       <c r="H8" s="0" t="n">
         <f aca="false">H6*H7/100</f>
-        <v>6016.38759043946</v>
+        <v>6313.223115874</v>
       </c>
       <c r="I8" s="0" t="n">
         <f aca="false">I6*I7/100</f>
-        <v>6287.12503200923</v>
+        <v>6565.75204050896</v>
       </c>
       <c r="J8" s="0" t="n">
         <f aca="false">J6*J7/100</f>
-        <v>6538.6100332896</v>
+        <v>6828.38212212932</v>
       </c>
       <c r="K8" s="0" t="n">
         <f aca="false">K6*K7/100</f>
-        <v>6734.76833428829</v>
+        <v>7067.37549640385</v>
       </c>
       <c r="L8" s="0" t="n">
         <f aca="false">L6*L7/100</f>
-        <v>6903.1375426455</v>
+        <v>7314.73363877798</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4609,43 +4609,43 @@
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Assumptions!D29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">Assumptions!E29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">Assumptions!F29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="G9" s="4" t="n">
         <f aca="false">Assumptions!G29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">Assumptions!H29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="I9" s="4" t="n">
         <f aca="false">Assumptions!I29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="J9" s="4" t="n">
         <f aca="false">Assumptions!J29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="K9" s="4" t="n">
         <f aca="false">Assumptions!K29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="L9" s="4" t="n">
         <f aca="false">Assumptions!L29</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4654,43 +4654,43 @@
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
-        <v>-52.456775</v>
+        <v>-74.910366</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">-D6*D9/100</f>
-        <v>-56.12874925</v>
+        <v>-78.6558843</v>
       </c>
       <c r="E10" s="0" t="n">
         <f aca="false">-E6*E9/100</f>
-        <v>-59.77711795125</v>
+        <v>-82.588678515</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">-F6*F9/100</f>
-        <v>-63.363745028325</v>
+        <v>-86.71811244075</v>
       </c>
       <c r="G10" s="0" t="n">
         <f aca="false">-G6*G9/100</f>
-        <v>-66.8487510048829</v>
+        <v>-90.6204275005838</v>
       </c>
       <c r="H10" s="0" t="n">
         <f aca="false">-H6*H9/100</f>
-        <v>-70.191188555127</v>
+        <v>-94.69834673811</v>
       </c>
       <c r="I10" s="0" t="n">
         <f aca="false">-I6*I9/100</f>
-        <v>-73.3497920401077</v>
+        <v>-98.4862806076344</v>
       </c>
       <c r="J10" s="0" t="n">
         <f aca="false">-J6*J9/100</f>
-        <v>-76.283783721712</v>
+        <v>-102.42573183194</v>
       </c>
       <c r="K10" s="0" t="n">
         <f aca="false">-K6*K9/100</f>
-        <v>-78.5722972333634</v>
+        <v>-106.010632446058</v>
       </c>
       <c r="L10" s="0" t="n">
         <f aca="false">-L6*L9/100</f>
-        <v>-80.5366046641975</v>
+        <v>-109.72100458167</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4699,43 +4699,43 @@
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
-        <v>4069.146975</v>
+        <v>4336.477854</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">D8+D10+D24</f>
-        <v>4434.17119075</v>
+        <v>4728.0926007</v>
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">E8+E10+E24</f>
-        <v>4807.78820093625</v>
+        <v>5148.027627435</v>
       </c>
       <c r="F11" s="0" t="n">
         <f aca="false">F8+F10+F24</f>
-        <v>5186.77512874718</v>
+        <v>5501.78246707425</v>
       </c>
       <c r="G11" s="0" t="n">
         <f aca="false">G8+G10+G24</f>
-        <v>5567.54597654953</v>
+        <v>5850.05204198213</v>
       </c>
       <c r="H11" s="0" t="n">
         <f aca="false">H8+H10+H24</f>
-        <v>5946.19640188433</v>
+        <v>6218.52476913589</v>
       </c>
       <c r="I11" s="0" t="n">
         <f aca="false">I8+I10+I24</f>
-        <v>6213.77523996913</v>
+        <v>6467.26575990133</v>
       </c>
       <c r="J11" s="0" t="n">
         <f aca="false">J8+J10+J24</f>
-        <v>6462.32624956789</v>
+        <v>6725.95639029738</v>
       </c>
       <c r="K11" s="0" t="n">
         <f aca="false">K8+K10+K24</f>
-        <v>6656.19603705493</v>
+        <v>6961.36486395779</v>
       </c>
       <c r="L11" s="0" t="n">
         <f aca="false">L8+L10+L24</f>
-        <v>6822.6009379813</v>
+        <v>7205.01263419631</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4744,43 +4744,43 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C31/100</f>
-        <v>-1124.07375</v>
+        <v>-1331.73984</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">-D6*Assumptions!D31/100</f>
-        <v>-1170.6853415</v>
+        <v>-1310.931405</v>
       </c>
       <c r="E12" s="4" t="n">
         <f aca="false">-E6*Assumptions!E31/100</f>
-        <v>-1212.6215355825</v>
+        <v>-1284.7127769</v>
       </c>
       <c r="F12" s="4" t="n">
         <f aca="false">-F6*Assumptions!F31/100</f>
-        <v>-1249.17097341555</v>
+        <v>-1252.5949574775</v>
       </c>
       <c r="G12" s="4" t="n">
         <f aca="false">-G6*Assumptions!G31/100</f>
-        <v>-1279.6760906649</v>
+        <v>-1208.27236667445</v>
       </c>
       <c r="H12" s="4" t="n">
         <f aca="false">-H6*Assumptions!H31/100</f>
-        <v>-1303.55064459522</v>
+        <v>-1052.20385264567</v>
       </c>
       <c r="I12" s="4" t="n">
         <f aca="false">-I6*Assumptions!I31/100</f>
-        <v>-1320.29625672194</v>
+        <v>-875.433605401195</v>
       </c>
       <c r="J12" s="4" t="n">
         <f aca="false">-J6*Assumptions!J31/100</f>
-        <v>-1351.31274021318</v>
+        <v>-682.838212212932</v>
       </c>
       <c r="K12" s="4" t="n">
         <f aca="false">-K6*Assumptions!K31/100</f>
-        <v>-1369.40289463862</v>
+        <v>-471.158366426923</v>
       </c>
       <c r="L12" s="4" t="n">
         <f aca="false">-L6*Assumptions!L31/100</f>
-        <v>-1380.6275085291</v>
+        <v>-268.206900088526</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4789,43 +4789,43 @@
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
-        <v>2945.073225</v>
+        <v>3004.738014</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">D11+D12</f>
-        <v>3263.48584925</v>
+        <v>3417.1611957</v>
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">E11+E12</f>
-        <v>3595.16666535375</v>
+        <v>3863.314850535</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">F11+F12</f>
-        <v>3937.60415533163</v>
+        <v>4249.18750959675</v>
       </c>
       <c r="G13" s="0" t="n">
         <f aca="false">G11+G12</f>
-        <v>4287.86988588463</v>
+        <v>4641.77967530768</v>
       </c>
       <c r="H13" s="0" t="n">
         <f aca="false">H11+H12</f>
-        <v>4642.64575728912</v>
+        <v>5166.32091649023</v>
       </c>
       <c r="I13" s="0" t="n">
         <f aca="false">I11+I12</f>
-        <v>4893.47898324719</v>
+        <v>5591.83215450013</v>
       </c>
       <c r="J13" s="0" t="n">
         <f aca="false">J11+J12</f>
-        <v>5111.01350935471</v>
+        <v>6043.11817808445</v>
       </c>
       <c r="K13" s="0" t="n">
         <f aca="false">K11+K12</f>
-        <v>5286.79314241631</v>
+        <v>6490.20649753087</v>
       </c>
       <c r="L13" s="0" t="n">
         <f aca="false">L11+L12</f>
-        <v>5441.9734294522</v>
+        <v>6936.80573410778</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4834,43 +4834,43 @@
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C33</f>
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="D14" s="4" t="n">
         <f aca="false">Assumptions!D33</f>
-        <v>19.5</v>
+        <v>24</v>
       </c>
       <c r="E14" s="4" t="n">
         <f aca="false">Assumptions!E33</f>
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F14" s="4" t="n">
         <f aca="false">Assumptions!F33</f>
-        <v>20.5</v>
+        <v>24</v>
       </c>
       <c r="G14" s="4" t="n">
         <f aca="false">Assumptions!G33</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H14" s="4" t="n">
         <f aca="false">Assumptions!H33</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I14" s="4" t="n">
         <f aca="false">Assumptions!I33</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J14" s="4" t="n">
         <f aca="false">Assumptions!J33</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K14" s="4" t="n">
         <f aca="false">Assumptions!K33</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="L14" s="4" t="n">
         <f aca="false">Assumptions!L33</f>
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4879,43 +4879,43 @@
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
-        <v>2385.50931225</v>
+        <v>2283.60089064</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">D13-MAX(0,D13)*D14/100</f>
-        <v>2627.10610864625</v>
+        <v>2597.042508732</v>
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">E13-MAX(0,E13)*E14/100</f>
-        <v>2876.133332283</v>
+        <v>2936.1192864066</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">F13-MAX(0,F13)*F14/100</f>
-        <v>3130.39530348864</v>
+        <v>3229.38250729353</v>
       </c>
       <c r="G15" s="0" t="n">
         <f aca="false">G13-MAX(0,G13)*G14/100</f>
-        <v>3387.41720984886</v>
+        <v>3527.75255323384</v>
       </c>
       <c r="H15" s="0" t="n">
         <f aca="false">H13-MAX(0,H13)*H14/100</f>
-        <v>3667.6901482584</v>
+        <v>3926.40389653257</v>
       </c>
       <c r="I15" s="0" t="n">
         <f aca="false">I13-MAX(0,I13)*I14/100</f>
-        <v>3865.84839676528</v>
+        <v>4249.7924374201</v>
       </c>
       <c r="J15" s="0" t="n">
         <f aca="false">J13-MAX(0,J13)*J14/100</f>
-        <v>4037.70067239022</v>
+        <v>4592.76981534418</v>
       </c>
       <c r="K15" s="0" t="n">
         <f aca="false">K13-MAX(0,K13)*K14/100</f>
-        <v>4176.56658250888</v>
+        <v>4932.55693812346</v>
       </c>
       <c r="L15" s="0" t="n">
         <f aca="false">L13-MAX(0,L13)*L14/100</f>
-        <v>4299.15900926724</v>
+        <v>5271.97235792192</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4924,43 +4924,43 @@
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
-        <v>1124.07375</v>
+        <v>1331.73984</v>
       </c>
       <c r="D16" s="0" t="n">
         <f aca="false">-D12</f>
-        <v>1170.6853415</v>
+        <v>1310.931405</v>
       </c>
       <c r="E16" s="0" t="n">
         <f aca="false">-E12</f>
-        <v>1212.6215355825</v>
+        <v>1284.7127769</v>
       </c>
       <c r="F16" s="0" t="n">
         <f aca="false">-F12</f>
-        <v>1249.17097341555</v>
+        <v>1252.5949574775</v>
       </c>
       <c r="G16" s="0" t="n">
         <f aca="false">-G12</f>
-        <v>1279.6760906649</v>
+        <v>1208.27236667445</v>
       </c>
       <c r="H16" s="0" t="n">
         <f aca="false">-H12</f>
-        <v>1303.55064459522</v>
+        <v>1052.20385264567</v>
       </c>
       <c r="I16" s="0" t="n">
         <f aca="false">-I12</f>
-        <v>1320.29625672194</v>
+        <v>875.433605401195</v>
       </c>
       <c r="J16" s="0" t="n">
         <f aca="false">-J12</f>
-        <v>1351.31274021318</v>
+        <v>682.838212212932</v>
       </c>
       <c r="K16" s="0" t="n">
         <f aca="false">-K12</f>
-        <v>1369.40289463862</v>
+        <v>471.158366426923</v>
       </c>
       <c r="L16" s="0" t="n">
         <f aca="false">-L12</f>
-        <v>1380.6275085291</v>
+        <v>268.206900088526</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4969,43 +4969,43 @@
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C32/100</f>
-        <v>-179.8518</v>
+        <v>-183.114228</v>
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">-D6*Assumptions!D32/100</f>
-        <v>-184.42303325</v>
+        <v>-192.2699394</v>
       </c>
       <c r="E17" s="4" t="n">
         <f aca="false">-E6*Assumptions!E32/100</f>
-        <v>-187.8709421325</v>
+        <v>-201.88343637</v>
       </c>
       <c r="F17" s="4" t="n">
         <f aca="false">-F6*Assumptions!F32/100</f>
-        <v>-199.14319866045</v>
+        <v>-211.9776081885</v>
       </c>
       <c r="G17" s="4" t="n">
         <f aca="false">-G6*Assumptions!G32/100</f>
-        <v>-200.546253014649</v>
+        <v>-221.516600556983</v>
       </c>
       <c r="H17" s="4" t="n">
         <f aca="false">-H6*Assumptions!H32/100</f>
-        <v>-210.573565665381</v>
+        <v>-231.484847582047</v>
       </c>
       <c r="I17" s="4" t="n">
         <f aca="false">-I6*Assumptions!I32/100</f>
-        <v>-209.570834400308</v>
+        <v>-240.744241485329</v>
       </c>
       <c r="J17" s="4" t="n">
         <f aca="false">-J6*Assumptions!J32/100</f>
-        <v>-217.95366777632</v>
+        <v>-250.374011144742</v>
       </c>
       <c r="K17" s="4" t="n">
         <f aca="false">-K6*Assumptions!K32/100</f>
-        <v>-224.49227780961</v>
+        <v>-259.137101534808</v>
       </c>
       <c r="L17" s="4" t="n">
         <f aca="false">-L6*Assumptions!L32/100</f>
-        <v>-230.10458475485</v>
+        <v>-268.206900088526</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5059,43 +5059,43 @@
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
-        <v>3329.73126225</v>
+        <v>3432.22650264</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">D15+D16+D17+D18</f>
-        <v>3613.36841689625</v>
+        <v>3715.703974332</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">E15+E16+E17+E18</f>
-        <v>3900.883925733</v>
+        <v>4018.9486269366</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">F15+F16+F17+F18</f>
-        <v>4180.42307824374</v>
+        <v>4269.99985658253</v>
       </c>
       <c r="G19" s="0" t="n">
         <f aca="false">G15+G16+G17+G18</f>
-        <v>4466.54704749911</v>
+        <v>4514.5083193513</v>
       </c>
       <c r="H19" s="0" t="n">
         <f aca="false">H15+H16+H17+H18</f>
-        <v>4760.66722718824</v>
+        <v>4747.12290159619</v>
       </c>
       <c r="I19" s="0" t="n">
         <f aca="false">I15+I16+I17+I18</f>
-        <v>4976.57381908691</v>
+        <v>4884.48180133597</v>
       </c>
       <c r="J19" s="0" t="n">
         <f aca="false">J15+J16+J17+J18</f>
-        <v>5171.05974482708</v>
+        <v>5025.23401641237</v>
       </c>
       <c r="K19" s="0" t="n">
         <f aca="false">K15+K16+K17+K18</f>
-        <v>5321.47719933789</v>
+        <v>5144.57820301557</v>
       </c>
       <c r="L19" s="0" t="n">
         <f aca="false">L15+L16+L17+L18</f>
-        <v>5449.68193304149</v>
+        <v>5271.97235792192</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5104,43 +5104,43 @@
       </c>
       <c r="C20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^C4</f>
-        <v>0.921658986175115</v>
+        <v>0.925925925925926</v>
       </c>
       <c r="D20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^D4</f>
-        <v>0.849455286797341</v>
+        <v>0.857338820301783</v>
       </c>
       <c r="E20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^E4</f>
-        <v>0.782908098430729</v>
+        <v>0.79383224102017</v>
       </c>
       <c r="F20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^F4</f>
-        <v>0.721574284267953</v>
+        <v>0.735029852796453</v>
       </c>
       <c r="G20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^G4</f>
-        <v>0.665045423288436</v>
+        <v>0.680583197033753</v>
       </c>
       <c r="H20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^H4</f>
-        <v>0.612945090588421</v>
+        <v>0.630169626883105</v>
       </c>
       <c r="I20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^I4</f>
-        <v>0.564926350772738</v>
+        <v>0.583490395262134</v>
       </c>
       <c r="J20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^J4</f>
-        <v>0.520669447716809</v>
+        <v>0.540268884501976</v>
       </c>
       <c r="K20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^K4</f>
-        <v>0.479879675315031</v>
+        <v>0.500248967131459</v>
       </c>
       <c r="L20" s="0" t="n">
         <f aca="false">1/(1+$B$27/100)^L4</f>
-        <v>0.442285415036895</v>
+        <v>0.463193488084684</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5149,43 +5149,43 @@
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
-        <v>3068.87673940092</v>
+        <v>3177.98750244444</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">D19*D20</f>
-        <v>3069.39490487906</v>
+        <v>3185.61726194444</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">E19*E20</f>
-        <v>3054.03361649462</v>
+        <v>3190.37099506602</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">F19*F20</f>
-        <v>3016.48579062096</v>
+        <v>3138.57736602473</v>
       </c>
       <c r="G21" s="0" t="n">
         <f aca="false">G19*G20</f>
-        <v>2970.45667184176</v>
+        <v>3072.49850501958</v>
       </c>
       <c r="H21" s="0" t="n">
         <f aca="false">H19*H20</f>
-        <v>2918.02760483022</v>
+        <v>2991.49266766711</v>
       </c>
       <c r="I21" s="0" t="n">
         <f aca="false">I19*I20</f>
-        <v>2811.39768696791</v>
+        <v>2850.04821691222</v>
       </c>
       <c r="J21" s="0" t="n">
         <f aca="false">J19*J20</f>
-        <v>2692.41282144974</v>
+        <v>2714.97757640849</v>
       </c>
       <c r="K21" s="0" t="n">
         <f aca="false">K19*K20</f>
-        <v>2553.66875061461</v>
+        <v>2573.56993238556</v>
       </c>
       <c r="L21" s="0" t="n">
         <f aca="false">L19*L20</f>
-        <v>2410.31483557433</v>
+        <v>2441.94326555189</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5289,7 +5289,7 @@
       </c>
       <c r="B27" s="4" t="n">
         <f aca="false">Assumptions!$B$34</f>
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5298,7 +5298,7 @@
       </c>
       <c r="B28" s="4" t="n">
         <f aca="false">Assumptions!$B$35</f>
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5307,7 +5307,7 @@
       </c>
       <c r="B29" s="4" t="n">
         <f aca="false">Assumptions!$B$36</f>
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
-        <v>28565.0694226741</v>
+        <v>29337.0832894245</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5325,7 +5325,7 @@
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
-        <v>5449.68193304149</v>
+        <v>5271.97235792192</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
-        <v>93098.7330227921</v>
+        <v>108602.630573191</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5343,7 +5343,7 @@
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
-        <v>98094.2747947468</v>
+        <v>105439.447158438</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5352,7 +5352,7 @@
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
-        <v>93098.7330227921</v>
+        <v>105439.447158438</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5361,7 +5361,7 @@
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
-        <v>41176.2117743947</v>
+        <v>48838.8653110378</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5370,7 +5370,7 @@
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
-        <v>69741.2811970689</v>
+        <v>78175.9486004623</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5379,7 +5379,7 @@
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
-        <v>59172.2811970689</v>
+        <v>65603.9486004623</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5388,7 +5388,7 @@
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>230.871171272216</v>
+        <v>253.004043966303</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5397,7 +5397,7 @@
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>0.0164714976983031</v>
+        <v>0.113917333537193</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5406,7 +5406,7 @@
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
-        <v>430.50983989622</v>
+        <v>604.105911216656</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5415,7 +5415,7 @@
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
-        <v>608.511162667602</v>
+        <v>1046.93432946379</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5424,7 +5424,7 @@
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>234.925096370007</v>
+        <v>259.371341462178</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5442,7 +5442,7 @@
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
-        <v>44687.3918509402</v>
+        <v>45251.0960721631</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5451,7 +5451,7 @@
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>84.8991846408731</v>
+        <v>77.2573751067425</v>
       </c>
     </row>
   </sheetData>
@@ -5573,35 +5573,35 @@
       </c>
       <c r="C5" s="4" t="n">
         <f aca="false">Assumptions!C41</f>
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">Assumptions!D41</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">Assumptions!E41</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">Assumptions!F41</f>
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="G5" s="4" t="n">
         <f aca="false">Assumptions!G41</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H5" s="4" t="n">
         <f aca="false">Assumptions!H41</f>
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="I5" s="4" t="n">
         <f aca="false">Assumptions!I41</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J5" s="4" t="n">
         <f aca="false">Assumptions!J41</f>
-        <v>5</v>
+        <v>4.5</v>
       </c>
       <c r="K5" s="4" t="n">
         <f aca="false">Assumptions!K41</f>
@@ -5609,7 +5609,7 @@
       </c>
       <c r="L5" s="4" t="n">
         <f aca="false">Assumptions!L41</f>
-        <v>3</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5621,43 +5621,43 @@
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">B6*(1+C5/100)</f>
-        <v>15336.2</v>
+        <v>16730.4</v>
       </c>
       <c r="D6" s="0" t="n">
         <f aca="false">C6*(1+D5/100)</f>
-        <v>16716.458</v>
+        <v>17901.528</v>
       </c>
       <c r="E6" s="0" t="n">
         <f aca="false">D6*(1+E5/100)</f>
-        <v>18053.77464</v>
+        <v>19154.63496</v>
       </c>
       <c r="F6" s="0" t="n">
         <f aca="false">E6*(1+F5/100)</f>
-        <v>19407.807738</v>
+        <v>20399.6862324</v>
       </c>
       <c r="G6" s="0" t="n">
         <f aca="false">F6*(1+G5/100)</f>
-        <v>20766.35427966</v>
+        <v>21623.667406344</v>
       </c>
       <c r="H6" s="0" t="n">
         <f aca="false">G6*(1+H5/100)</f>
-        <v>22116.1673078379</v>
+        <v>22812.9691136929</v>
       </c>
       <c r="I6" s="0" t="n">
         <f aca="false">H6*(1+I5/100)</f>
-        <v>23443.1373463082</v>
+        <v>23953.6175693776</v>
       </c>
       <c r="J6" s="0" t="n">
         <f aca="false">I6*(1+J5/100)</f>
-        <v>24615.2942136236</v>
+        <v>25031.5303599996</v>
       </c>
       <c r="K6" s="0" t="n">
         <f aca="false">J6*(1+K5/100)</f>
-        <v>25599.9059821685</v>
+        <v>26032.7915743995</v>
       </c>
       <c r="L6" s="0" t="n">
         <f aca="false">K6*(1+L5/100)</f>
-        <v>26367.9031616336</v>
+        <v>26943.9392795035</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5666,43 +5666,43 @@
       </c>
       <c r="C7" s="4" t="n">
         <f aca="false">Assumptions!C42</f>
-        <v>28.5</v>
+        <v>27</v>
       </c>
       <c r="D7" s="4" t="n">
         <f aca="false">Assumptions!D42</f>
-        <v>29.5</v>
+        <v>28.5</v>
       </c>
       <c r="E7" s="4" t="n">
         <f aca="false">Assumptions!E42</f>
-        <v>30.5</v>
+        <v>29.5</v>
       </c>
       <c r="F7" s="4" t="n">
         <f aca="false">Assumptions!F42</f>
-        <v>31.5</v>
+        <v>30.5</v>
       </c>
       <c r="G7" s="4" t="n">
         <f aca="false">Assumptions!G42</f>
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="H7" s="4" t="n">
         <f aca="false">Assumptions!H42</f>
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="I7" s="4" t="n">
         <f aca="false">Assumptions!I42</f>
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="J7" s="4" t="n">
         <f aca="false">Assumptions!J42</f>
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="K7" s="4" t="n">
         <f aca="false">Assumptions!K42</f>
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="L7" s="4" t="n">
         <f aca="false">Assumptions!L42</f>
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5711,43 +5711,43 @@
       </c>
       <c r="C8" s="0" t="n">
         <f aca="false">C6*C7/100</f>
-        <v>4370.817</v>
+        <v>4517.208</v>
       </c>
       <c r="D8" s="0" t="n">
         <f aca="false">D6*D7/100</f>
-        <v>4931.35511</v>
+        <v>5101.93548</v>
       </c>
       <c r="E8" s="0" t="n">
         <f aca="false">E6*E7/100</f>
-        <v>5506.4012652</v>
+        <v>5650.6173132</v>
       </c>
       <c r="F8" s="0" t="n">
         <f aca="false">F6*F7/100</f>
-        <v>6113.45943747</v>
+        <v>6221.904300882</v>
       </c>
       <c r="G8" s="0" t="n">
         <f aca="false">G6*G7/100</f>
-        <v>6645.2333694912</v>
+        <v>6703.33689596664</v>
       </c>
       <c r="H8" s="0" t="n">
         <f aca="false">H6*H7/100</f>
-        <v>7187.75437504732</v>
+        <v>7186.08527081327</v>
       </c>
       <c r="I8" s="0" t="n">
         <f aca="false">I6*I7/100</f>
-        <v>7619.01963755016</v>
+        <v>7545.38953435393</v>
       </c>
       <c r="J8" s="0" t="n">
         <f aca="false">J6*J7/100</f>
-        <v>7999.97061942767</v>
+        <v>7884.93206339986</v>
       </c>
       <c r="K8" s="0" t="n">
         <f aca="false">K6*K7/100</f>
-        <v>8319.96944420477</v>
+        <v>8200.32934593585</v>
       </c>
       <c r="L8" s="0" t="n">
         <f aca="false">L6*L7/100</f>
-        <v>8569.56852753092</v>
+        <v>8487.34087304361</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5756,43 +5756,43 @@
       </c>
       <c r="C9" s="4" t="n">
         <f aca="false">Assumptions!C43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="D9" s="4" t="n">
         <f aca="false">Assumptions!D43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="E9" s="4" t="n">
         <f aca="false">Assumptions!E43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="F9" s="4" t="n">
         <f aca="false">Assumptions!F43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="G9" s="4" t="n">
         <f aca="false">Assumptions!G43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="H9" s="4" t="n">
         <f aca="false">Assumptions!H43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="I9" s="4" t="n">
         <f aca="false">Assumptions!I43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="J9" s="4" t="n">
         <f aca="false">Assumptions!J43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="K9" s="4" t="n">
         <f aca="false">Assumptions!K43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
       <c r="L9" s="4" t="n">
         <f aca="false">Assumptions!L43</f>
-        <v>0.35</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5801,43 +5801,43 @@
       </c>
       <c r="C10" s="0" t="n">
         <f aca="false">-C6*C9/100</f>
-        <v>-53.6767</v>
+        <v>-75.2868</v>
       </c>
       <c r="D10" s="0" t="n">
         <f aca="false">-D6*D9/100</f>
-        <v>-58.507603</v>
+        <v>-80.556876</v>
       </c>
       <c r="E10" s="0" t="n">
         <f aca="false">-E6*E9/100</f>
-        <v>-63.18821124</v>
+        <v>-86.19585732</v>
       </c>
       <c r="F10" s="0" t="n">
         <f aca="false">-F6*F9/100</f>
-        <v>-67.927327083</v>
+        <v>-91.7985880458</v>
       </c>
       <c r="G10" s="0" t="n">
         <f aca="false">-G6*G9/100</f>
-        <v>-72.68223997881</v>
+        <v>-97.306503328548</v>
       </c>
       <c r="H10" s="0" t="n">
         <f aca="false">-H6*H9/100</f>
-        <v>-77.4065855774327</v>
+        <v>-102.658361011618</v>
       </c>
       <c r="I10" s="0" t="n">
         <f aca="false">-I6*I9/100</f>
-        <v>-82.0509807120786</v>
+        <v>-107.791279062199</v>
       </c>
       <c r="J10" s="0" t="n">
         <f aca="false">-J6*J9/100</f>
-        <v>-86.1535297476826</v>
+        <v>-112.641886619998</v>
       </c>
       <c r="K10" s="0" t="n">
         <f aca="false">-K6*K9/100</f>
-        <v>-89.5996709375899</v>
+        <v>-117.147562084798</v>
       </c>
       <c r="L10" s="0" t="n">
         <f aca="false">-L6*L9/100</f>
-        <v>-92.2876610657175</v>
+        <v>-121.247726757766</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5846,43 +5846,43 @@
       </c>
       <c r="C11" s="0" t="n">
         <f aca="false">C8+C10+C24</f>
-        <v>4317.1403</v>
+        <v>4441.9212</v>
       </c>
       <c r="D11" s="0" t="n">
         <f aca="false">D8+D10+D24</f>
-        <v>4872.847507</v>
+        <v>5021.378604</v>
       </c>
       <c r="E11" s="0" t="n">
         <f aca="false">E8+E10+E24</f>
-        <v>5443.21305396</v>
+        <v>5564.42145588</v>
       </c>
       <c r="F11" s="0" t="n">
         <f aca="false">F8+F10+F24</f>
-        <v>6045.532110387</v>
+        <v>6130.1057128362</v>
       </c>
       <c r="G11" s="0" t="n">
         <f aca="false">G8+G10+G24</f>
-        <v>6572.55112951239</v>
+        <v>6606.03039263809</v>
       </c>
       <c r="H11" s="0" t="n">
         <f aca="false">H8+H10+H24</f>
-        <v>7110.34778946989</v>
+        <v>7083.42690980165</v>
       </c>
       <c r="I11" s="0" t="n">
         <f aca="false">I8+I10+I24</f>
-        <v>7536.96865683808</v>
+        <v>7437.59825529173</v>
       </c>
       <c r="J11" s="0" t="n">
         <f aca="false">J8+J10+J24</f>
-        <v>7913.81708967998</v>
+        <v>7772.29017677986</v>
       </c>
       <c r="K11" s="0" t="n">
         <f aca="false">K8+K10+K24</f>
-        <v>8230.36977326718</v>
+        <v>8083.18178385106</v>
       </c>
       <c r="L11" s="0" t="n">
         <f aca="false">L8+L10+L24</f>
-        <v>8477.2808664652</v>
+        <v>8366.09314628584</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5891,43 +5891,43 @@
       </c>
       <c r="C12" s="4" t="n">
         <f aca="false">-C6*Assumptions!C45/100</f>
-        <v>-1119.5426</v>
+        <v>-1338.432</v>
       </c>
       <c r="D12" s="4" t="n">
         <f aca="false">-D6*Assumptions!D45/100</f>
-        <v>-1170.15206</v>
+        <v>-1342.6146</v>
       </c>
       <c r="E12" s="4" t="n">
         <f aca="false">-E6*Assumptions!E45/100</f>
-        <v>-1209.60290088</v>
+        <v>-1340.8244472</v>
       </c>
       <c r="F12" s="4" t="n">
         <f aca="false">-F6*Assumptions!F45/100</f>
-        <v>-1242.099695232</v>
+        <v>-1325.979605106</v>
       </c>
       <c r="G12" s="4" t="n">
         <f aca="false">-G6*Assumptions!G45/100</f>
-        <v>-1266.74761105926</v>
+        <v>-1297.42004438064</v>
       </c>
       <c r="H12" s="4" t="n">
         <f aca="false">-H6*Assumptions!H45/100</f>
-        <v>-1304.85387116244</v>
+        <v>-1140.64845568465</v>
       </c>
       <c r="I12" s="4" t="n">
         <f aca="false">-I6*Assumptions!I45/100</f>
-        <v>-1336.25882873957</v>
+        <v>-958.144702775103</v>
       </c>
       <c r="J12" s="4" t="n">
         <f aca="false">-J6*Assumptions!J45/100</f>
-        <v>-1353.8411817493</v>
+        <v>-750.945910799987</v>
       </c>
       <c r="K12" s="4" t="n">
         <f aca="false">-K6*Assumptions!K45/100</f>
-        <v>-1382.3949230371</v>
+        <v>-520.655831487991</v>
       </c>
       <c r="L12" s="4" t="n">
         <f aca="false">-L6*Assumptions!L45/100</f>
-        <v>-1397.49886756658</v>
+        <v>-296.383332074539</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5936,43 +5936,43 @@
       </c>
       <c r="C13" s="0" t="n">
         <f aca="false">C11+C12</f>
-        <v>3197.5977</v>
+        <v>3103.4892</v>
       </c>
       <c r="D13" s="0" t="n">
         <f aca="false">D11+D12</f>
-        <v>3702.695447</v>
+        <v>3678.764004</v>
       </c>
       <c r="E13" s="0" t="n">
         <f aca="false">E11+E12</f>
-        <v>4233.61015308</v>
+        <v>4223.59700868</v>
       </c>
       <c r="F13" s="0" t="n">
         <f aca="false">F11+F12</f>
-        <v>4803.432415155</v>
+        <v>4804.1261077302</v>
       </c>
       <c r="G13" s="0" t="n">
         <f aca="false">G11+G12</f>
-        <v>5305.80351845313</v>
+        <v>5308.61034825745</v>
       </c>
       <c r="H13" s="0" t="n">
         <f aca="false">H11+H12</f>
-        <v>5805.49391830745</v>
+        <v>5942.77845411701</v>
       </c>
       <c r="I13" s="0" t="n">
         <f aca="false">I11+I12</f>
-        <v>6200.70982809851</v>
+        <v>6479.45355251663</v>
       </c>
       <c r="J13" s="0" t="n">
         <f aca="false">J11+J12</f>
-        <v>6559.97590793069</v>
+        <v>7021.34426597988</v>
       </c>
       <c r="K13" s="0" t="n">
         <f aca="false">K11+K12</f>
-        <v>6847.97485023008</v>
+        <v>7562.52595236307</v>
       </c>
       <c r="L13" s="0" t="n">
         <f aca="false">L11+L12</f>
-        <v>7079.78199889862</v>
+        <v>8069.7098142113</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5981,43 +5981,43 @@
       </c>
       <c r="C14" s="4" t="n">
         <f aca="false">Assumptions!C47</f>
-        <v>18.5</v>
+        <v>24</v>
       </c>
       <c r="D14" s="4" t="n">
         <f aca="false">Assumptions!D47</f>
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="E14" s="4" t="n">
         <f aca="false">Assumptions!E47</f>
-        <v>19.5</v>
+        <v>24</v>
       </c>
       <c r="F14" s="4" t="n">
         <f aca="false">Assumptions!F47</f>
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G14" s="4" t="n">
         <f aca="false">Assumptions!G47</f>
-        <v>20.5</v>
+        <v>24</v>
       </c>
       <c r="H14" s="4" t="n">
         <f aca="false">Assumptions!H47</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I14" s="4" t="n">
         <f aca="false">Assumptions!I47</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="J14" s="4" t="n">
         <f aca="false">Assumptions!J47</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="K14" s="4" t="n">
         <f aca="false">Assumptions!K47</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="L14" s="4" t="n">
         <f aca="false">Assumptions!L47</f>
-        <v>21</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6026,43 +6026,43 @@
       </c>
       <c r="C15" s="0" t="n">
         <f aca="false">C13-MAX(0,C13)*C14/100</f>
-        <v>2606.0421255</v>
+        <v>2358.651792</v>
       </c>
       <c r="D15" s="0" t="n">
         <f aca="false">D13-MAX(0,D13)*D14/100</f>
-        <v>2999.18331207</v>
+        <v>2795.86064304</v>
       </c>
       <c r="E15" s="0" t="n">
         <f aca="false">E13-MAX(0,E13)*E14/100</f>
-        <v>3408.0561732294</v>
+        <v>3209.9337265968</v>
       </c>
       <c r="F15" s="0" t="n">
         <f aca="false">F13-MAX(0,F13)*F14/100</f>
-        <v>3842.745932124</v>
+        <v>3651.13584187495</v>
       </c>
       <c r="G15" s="0" t="n">
         <f aca="false">G13-MAX(0,G13)*G14/100</f>
-        <v>4218.11379717024</v>
+        <v>4034.54386467566</v>
       </c>
       <c r="H15" s="0" t="n">
         <f aca="false">H13-MAX(0,H13)*H14/100</f>
-        <v>4586.34019546289</v>
+        <v>4516.51162512893</v>
       </c>
       <c r="I15" s="0" t="n">
         <f aca="false">I13-MAX(0,I13)*I14/100</f>
-        <v>4898.56076419782</v>
+        <v>4924.38469991264</v>
       </c>
       <c r="J15" s="0" t="n">
         <f aca="false">J13-MAX(0,J13)*J14/100</f>
-        <v>5182.38096726524</v>
+        <v>5336.22164214471</v>
       </c>
       <c r="K15" s="0" t="n">
         <f aca="false">K13-MAX(0,K13)*K14/100</f>
-        <v>5409.90013168177</v>
+        <v>5747.51972379593</v>
       </c>
       <c r="L15" s="0" t="n">
         <f aca="false">L13-MAX(0,L13)*L14/100</f>
-        <v>5593.02777912991</v>
+        <v>6132.97945880059</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6071,43 +6071,43 @@
       </c>
       <c r="C16" s="0" t="n">
         <f aca="false">-C12</f>
-        <v>1119.5426</v>
+        <v>1338.432</v>
       </c>
       <c r="D16" s="0" t="n">
         <f aca="false">-D12</f>
-        <v>1170.15206</v>
+        <v>1342.6146</v>
       </c>
       <c r="E16" s="0" t="n">
         <f aca="false">-E12</f>
-        <v>1209.60290088</v>
+        <v>1340.8244472</v>
       </c>
       <c r="F16" s="0" t="n">
         <f aca="false">-F12</f>
-        <v>1242.099695232</v>
+        <v>1325.979605106</v>
       </c>
       <c r="G16" s="0" t="n">
         <f aca="false">-G12</f>
-        <v>1266.74761105926</v>
+        <v>1297.42004438064</v>
       </c>
       <c r="H16" s="0" t="n">
         <f aca="false">-H12</f>
-        <v>1304.85387116244</v>
+        <v>1140.64845568465</v>
       </c>
       <c r="I16" s="0" t="n">
         <f aca="false">-I12</f>
-        <v>1336.25882873957</v>
+        <v>958.144702775103</v>
       </c>
       <c r="J16" s="0" t="n">
         <f aca="false">-J12</f>
-        <v>1353.8411817493</v>
+        <v>750.945910799987</v>
       </c>
       <c r="K16" s="0" t="n">
         <f aca="false">-K12</f>
-        <v>1382.3949230371</v>
+        <v>520.655831487991</v>
       </c>
       <c r="L16" s="0" t="n">
         <f aca="false">-L12</f>
-        <v>1397.49886756658</v>
+        <v>296.383332074539</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6116,43 +6116,43 @@
       </c>
       <c r="C17" s="4" t="n">
         <f aca="false">-C6*Assumptions!C46/100</f>
-        <v>-176.3663</v>
+        <v>-184.0344</v>
       </c>
       <c r="D17" s="4" t="n">
         <f aca="false">-D6*Assumptions!D46/100</f>
-        <v>-183.881038</v>
+        <v>-196.916808</v>
       </c>
       <c r="E17" s="4" t="n">
         <f aca="false">-E6*Assumptions!E46/100</f>
-        <v>-189.56463372</v>
+        <v>-210.70098456</v>
       </c>
       <c r="F17" s="4" t="n">
         <f aca="false">-F6*Assumptions!F46/100</f>
-        <v>-194.07807738</v>
+        <v>-224.3965485564</v>
       </c>
       <c r="G17" s="4" t="n">
         <f aca="false">-G6*Assumptions!G46/100</f>
-        <v>-207.6635427966</v>
+        <v>-237.860341469784</v>
       </c>
       <c r="H17" s="4" t="n">
         <f aca="false">-H6*Assumptions!H46/100</f>
-        <v>-210.10358942446</v>
+        <v>-250.942660250622</v>
       </c>
       <c r="I17" s="4" t="n">
         <f aca="false">-I6*Assumptions!I46/100</f>
-        <v>-222.709804789928</v>
+        <v>-263.489793263153</v>
       </c>
       <c r="J17" s="4" t="n">
         <f aca="false">-J6*Assumptions!J46/100</f>
-        <v>-221.537647922612</v>
+        <v>-275.346833959995</v>
       </c>
       <c r="K17" s="4" t="n">
         <f aca="false">-K6*Assumptions!K46/100</f>
-        <v>-230.399153839517</v>
+        <v>-286.360707318395</v>
       </c>
       <c r="L17" s="4" t="n">
         <f aca="false">-L6*Assumptions!L46/100</f>
-        <v>-237.311128454702</v>
+        <v>-296.383332074539</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6206,43 +6206,43 @@
       </c>
       <c r="C19" s="0" t="n">
         <f aca="false">C15+C16+C17+C18</f>
-        <v>3549.2184255</v>
+        <v>3513.049392</v>
       </c>
       <c r="D19" s="0" t="n">
         <f aca="false">D15+D16+D17+D18</f>
-        <v>3985.45433407</v>
+        <v>3941.55843504</v>
       </c>
       <c r="E19" s="0" t="n">
         <f aca="false">E15+E16+E17+E18</f>
-        <v>4428.0944403894</v>
+        <v>4340.0571892368</v>
       </c>
       <c r="F19" s="0" t="n">
         <f aca="false">F15+F16+F17+F18</f>
-        <v>4890.767549976</v>
+        <v>4752.71889842455</v>
       </c>
       <c r="G19" s="0" t="n">
         <f aca="false">G15+G16+G17+G18</f>
-        <v>5277.1978654329</v>
+        <v>5094.10356758652</v>
       </c>
       <c r="H19" s="0" t="n">
         <f aca="false">H15+H16+H17+H18</f>
-        <v>5681.09047720086</v>
+        <v>5406.21742056295</v>
       </c>
       <c r="I19" s="0" t="n">
         <f aca="false">I15+I16+I17+I18</f>
-        <v>6012.10978814746</v>
+        <v>5619.03960942459</v>
       </c>
       <c r="J19" s="0" t="n">
         <f aca="false">J15+J16+J17+J18</f>
-        <v>6314.68450109193</v>
+        <v>5811.8207189847</v>
       </c>
       <c r="K19" s="0" t="n">
         <f aca="false">K15+K16+K17+K18</f>
-        <v>6561.89590087935</v>
+        <v>5981.81484796553</v>
       </c>
       <c r="L19" s="0" t="n">
         <f aca="false">L15+L16+L17+L18</f>
-        <v>6753.21551824179</v>
+        <v>6132.97945880059</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6296,43 +6296,43 @@
       </c>
       <c r="C21" s="0" t="n">
         <f aca="false">C19*C20</f>
-        <v>3286.31335694444</v>
+        <v>3252.82351111111</v>
       </c>
       <c r="D21" s="0" t="n">
         <f aca="false">D19*D20</f>
-        <v>3416.8847171382</v>
+        <v>3379.25105884774</v>
       </c>
       <c r="E21" s="0" t="n">
         <f aca="false">E19*E20</f>
-        <v>3515.16413306327</v>
+        <v>3445.27732468755</v>
       </c>
       <c r="F21" s="0" t="n">
         <f aca="false">F19*F20</f>
-        <v>3594.86015232053</v>
+        <v>3493.39027229192</v>
       </c>
       <c r="G21" s="0" t="n">
         <f aca="false">G19*G20</f>
-        <v>3591.57219463602</v>
+        <v>3466.96129204908</v>
       </c>
       <c r="H21" s="0" t="n">
         <f aca="false">H19*H20</f>
-        <v>3580.05066630683</v>
+        <v>3406.83401476509</v>
       </c>
       <c r="I21" s="0" t="n">
         <f aca="false">I19*I20</f>
-        <v>3508.00831664551</v>
+        <v>3278.65564269674</v>
       </c>
       <c r="J21" s="0" t="n">
         <f aca="false">J19*J20</f>
-        <v>3411.62755138685</v>
+        <v>3139.94589677133</v>
       </c>
       <c r="K21" s="0" t="n">
         <f aca="false">K19*K20</f>
-        <v>3282.58164683905</v>
+        <v>2992.39669926638</v>
       </c>
       <c r="L21" s="0" t="n">
         <f aca="false">L19*L20</f>
-        <v>3128.04545168203</v>
+        <v>2840.75614787356</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6463,7 +6463,7 @@
       </c>
       <c r="B30" s="0" t="n">
         <f aca="false">SUM(C21:L21)</f>
-        <v>34315.1081869627</v>
+        <v>32696.2918603605</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6472,7 +6472,7 @@
       </c>
       <c r="B31" s="0" t="n">
         <f aca="false">L19</f>
-        <v>6753.21551824179</v>
+        <v>6132.97945880059</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6481,7 +6481,7 @@
       </c>
       <c r="B32" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,B31*(1+B28/100)/((B27-B28)/100),B31*B29)</f>
-        <v>139116.239675781</v>
+        <v>126339.376851292</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6490,7 +6490,7 @@
       </c>
       <c r="B33" s="0" t="n">
         <f aca="false">B31*B29</f>
-        <v>135064.310364836</v>
+        <v>122659.589176012</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6499,7 +6499,7 @@
       </c>
       <c r="B34" s="0" t="n">
         <f aca="false">MAX(0,MIN(B32,B33))</f>
-        <v>135064.310364836</v>
+        <v>122659.589176012</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6508,7 +6508,7 @@
       </c>
       <c r="B35" s="0" t="n">
         <f aca="false">B34/(1+B27/100)^L4</f>
-        <v>62560.9090336406</v>
+        <v>56815.1229574713</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="B36" s="0" t="n">
         <f aca="false">B30+B35</f>
-        <v>96876.0172206034</v>
+        <v>89511.4148178318</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6526,7 +6526,7 @@
       </c>
       <c r="B37" s="0" t="n">
         <f aca="false">B36+Assumptions!$B$5-Assumptions!$B$4</f>
-        <v>86307.0172206034</v>
+        <v>76939.4148178318</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="B38" s="0" t="n">
         <f aca="false">B37/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>336.742166291859</v>
+        <v>296.719686917978</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6544,7 +6544,7 @@
       </c>
       <c r="B39" s="4" t="n">
         <f aca="false">B38/Assumptions!$B$2-1</f>
-        <v>0.482596602350454</v>
+        <v>0.30638703349614</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6553,7 +6553,7 @@
       </c>
       <c r="B41" s="0" t="n">
         <f aca="false">SUMPRODUCT(-C10:L10/(1+$B$27/100)^C4:L4)</f>
-        <v>480.187747506291</v>
+        <v>644.10782933325</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6562,7 +6562,7 @@
       </c>
       <c r="B42" s="0" t="n">
         <f aca="false">IF(B27&gt;B28,-L10*(1+B28/100)/((B27-B28)/100),-L10*20)/(1+B27/100)^L4</f>
-        <v>880.58909890586</v>
+        <v>1156.91984407293</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6571,7 +6571,7 @@
       </c>
       <c r="B43" s="0" t="n">
         <f aca="false">(B37+B41+B42)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>342.051478997329</v>
+        <v>303.665416472187</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6589,7 +6589,7 @@
       </c>
       <c r="B46" s="0" t="n">
         <f aca="false">MAX(0,MIN(IF(B45&gt;B28,B31*(1+B28/100)/((B45-B28)/100),B31*B29),B31*B29))</f>
-        <v>57965.0998649087</v>
+        <v>52641.4070213717</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6598,7 +6598,7 @@
       </c>
       <c r="B47" s="0" t="n">
         <f aca="false">(SUMPRODUCT(C19:L19/(1+B45/100)^C4:L4)+B46/(1+B45/100)^L4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>111.219804068549</v>
+        <v>93.1161259688547</v>
       </c>
     </row>
   </sheetData>
@@ -6654,23 +6654,23 @@
       </c>
       <c r="B4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$38</f>
-        <v>111.27041068658</v>
+        <v>168.39448756212</v>
       </c>
       <c r="C4" s="0" t="n">
         <f aca="false">B4/Assumptions!$B$2-1</f>
-        <v>-0.510102537372519</v>
+        <v>-0.258598654681811</v>
       </c>
       <c r="D4" s="4" t="n">
         <f aca="false">Assumptions!$B$24</f>
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="E4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$43</f>
-        <v>113.823707098543</v>
+        <v>174.413016509053</v>
       </c>
       <c r="F4" s="4" t="n">
         <f aca="false">DCF_Bear!$B$47</f>
-        <v>51.6192428477828</v>
+        <v>56.1173485238053</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6679,23 +6679,23 @@
       </c>
       <c r="B5" s="4" t="n">
         <f aca="false">DCF_Base!$B$38</f>
-        <v>230.871171272216</v>
+        <v>253.004043966303</v>
       </c>
       <c r="C5" s="0" t="n">
         <f aca="false">B5/Assumptions!$B$2-1</f>
-        <v>0.0164714976983031</v>
+        <v>0.113917333537193</v>
       </c>
       <c r="D5" s="4" t="n">
         <f aca="false">Assumptions!$B$38</f>
-        <v>0.5</v>
+        <v>0.55</v>
       </c>
       <c r="E5" s="4" t="n">
         <f aca="false">DCF_Base!$B$43</f>
-        <v>234.925096370007</v>
+        <v>259.371341462178</v>
       </c>
       <c r="F5" s="4" t="n">
         <f aca="false">DCF_Base!$B$47</f>
-        <v>84.8991846408731</v>
+        <v>77.2573751067425</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6704,11 +6704,11 @@
       </c>
       <c r="B6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$38</f>
-        <v>336.742166291859</v>
+        <v>296.719686917978</v>
       </c>
       <c r="C6" s="0" t="n">
         <f aca="false">B6/Assumptions!$B$2-1</f>
-        <v>0.482596602350454</v>
+        <v>0.30638703349614</v>
       </c>
       <c r="D6" s="4" t="n">
         <f aca="false">Assumptions!$B$52</f>
@@ -6716,11 +6716,11 @@
       </c>
       <c r="E6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$43</f>
-        <v>342.051478997329</v>
+        <v>303.665416472187</v>
       </c>
       <c r="F6" s="4" t="n">
         <f aca="false">DCF_Bull!$B$47</f>
-        <v>111.219804068549</v>
+        <v>93.1161259688547</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6729,7 +6729,7 @@
       </c>
       <c r="B8" s="0" t="n">
         <f aca="false">SUMPRODUCT(B4:B6,D4:D6)</f>
-        <v>227.438729880717</v>
+        <v>247.011043423385</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6738,7 +6738,7 @@
       </c>
       <c r="B9" s="0" t="n">
         <f aca="false">SUMPRODUCT(E4:E6,D4:D6)</f>
-        <v>231.431344708971</v>
+        <v>253.453195224055</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6747,7 +6747,7 @@
       </c>
       <c r="B10" s="0" t="n">
         <f aca="false">1-Assumptions!$B$2/B8</f>
-        <v>0.00135742000001193</v>
+        <v>0.0804864557788547</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6756,7 +6756,7 @@
       </c>
       <c r="B11" s="0" t="n">
         <f aca="false">IF(ABS(B9-B8)&gt;0.01*ABS(B8),(Assumptions!$B$2-B8)/(B9-B8)*100,"n/a")</f>
-        <v>-7.73252352149441</v>
+        <v>-308.60873879621</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6765,7 +6765,7 @@
       </c>
       <c r="B12" s="0" t="n">
         <f aca="false">SUMPRODUCT(F4:F6,D4:D6)</f>
-        <v>83.1593540495194</v>
+        <v>76.9940575056831</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6782,10 +6782,10 @@
       </c>
       <c r="B15" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$15/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$15&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$15-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$15/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>230.871171272216</v>
+        <v>253.004043966303</v>
       </c>
       <c r="C15" s="3" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6794,7 +6794,7 @@
       </c>
       <c r="B16" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$16/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$16&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$16-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$16/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>209.180382545203</v>
+        <v>206.772096835689</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>9</v>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="B17" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$17/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$17&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$17-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$17/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>174.521660189135</v>
+        <v>169.729446683243</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>10</v>
@@ -6818,7 +6818,7 @@
       </c>
       <c r="B18" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$18/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$18&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$18-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$18/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>148.069919800294</v>
+        <v>141.961347784994</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>11</v>
@@ -6830,7 +6830,7 @@
       </c>
       <c r="B19" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$19/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$19&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$19-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$19/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>127.230702307382</v>
+        <v>120.376001127906</v>
       </c>
       <c r="C19" s="3" t="n">
         <v>12</v>
@@ -6842,7 +6842,7 @@
       </c>
       <c r="B20" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$C$20/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($C$20&gt;DCF_Base!$B$28,DCF_Base!$L$19*(1+DCF_Base!$B$28/100)/(($C$20-DCF_Base!$B$28)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$C$20/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>84.8991846408731</v>
+        <v>77.2573751067425</v>
       </c>
       <c r="C20" s="3" t="n">
         <v>15</v>
@@ -6855,144 +6855,144 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="3" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D23" s="3" t="n">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="F23" s="3" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="B24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$24-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>285.80388607099</v>
+        <v>303.573762797355</v>
       </c>
       <c r="C24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$24-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>285.80388607099</v>
+        <v>303.573762797355</v>
       </c>
       <c r="D24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$24-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>285.80388607099</v>
+        <v>303.573762797355</v>
       </c>
       <c r="E24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$24-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>285.80388607099</v>
+        <v>303.573762797355</v>
       </c>
       <c r="F24" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$24/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$24&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$24-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$24/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>285.80388607099</v>
+        <v>303.573762797355</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="n">
-        <v>7.5</v>
+        <v>7</v>
       </c>
       <c r="B25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$25-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>250.372867108816</v>
+        <v>277.077760783172</v>
       </c>
       <c r="C25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$25-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>261.54921761152</v>
+        <v>277.077760783172</v>
       </c>
       <c r="D25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$25-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>261.54921761152</v>
+        <v>277.077760783172</v>
       </c>
       <c r="E25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$25-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>261.54921761152</v>
+        <v>277.077760783172</v>
       </c>
       <c r="F25" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$25/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$25&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$25-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$25/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>261.54921761152</v>
+        <v>277.077760783172</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="n">
-        <v>8.5</v>
+        <v>8</v>
       </c>
       <c r="B26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$26-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>206.576802725329</v>
+        <v>224.751711545725</v>
       </c>
       <c r="C26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$26-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>217.789588208507</v>
+        <v>240.162074684222</v>
       </c>
       <c r="D26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$26-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>230.871171272216</v>
+        <v>253.004043966303</v>
       </c>
       <c r="E26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$26-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>239.49175365982</v>
+        <v>253.004043966303</v>
       </c>
       <c r="F26" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$26/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$26&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$26-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$26/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>239.49175365982</v>
+        <v>253.004043966303</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="B27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$27-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>173.828336551241</v>
+        <v>184.483494495788</v>
       </c>
       <c r="C27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$27-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>181.657479647397</v>
+        <v>194.770541729589</v>
       </c>
       <c r="D27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$27-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>190.60507175729</v>
+        <v>206.772096835689</v>
       </c>
       <c r="E27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$27-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>200.929216499474</v>
+        <v>220.955752870172</v>
       </c>
       <c r="F27" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$27/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$27&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$27-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$27/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>212.974052032023</v>
+        <v>231.105525078334</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="n">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="B28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$B$23,DCF_Base!$L$19*(1+$B$23/100)/(($A$28-$B$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>148.439018069074</v>
+        <v>154.332010446119</v>
       </c>
       <c r="C28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$C$23,DCF_Base!$L$19*(1+$C$23/100)/(($A$28-$C$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>154.097118039254</v>
+        <v>161.51748069011</v>
       </c>
       <c r="D28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$D$23,DCF_Base!$L$19*(1+$D$23/100)/(($A$28-$D$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>160.462480505706</v>
+        <v>169.729446683243</v>
       </c>
       <c r="E28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$E$23,DCF_Base!$L$19*(1+$E$23/100)/(($A$28-$E$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>167.676557967685</v>
+        <v>179.204792059935</v>
       </c>
       <c r="F28" s="0" t="n">
         <f aca="false">(SUMPRODUCT(DCF_Base!$C$19:$L$19/(1+$A$28/100)^DCF_Base!$C$4:$L$4)+MAX(0,MIN(IF($A$28&gt;$F$23,DCF_Base!$L$19*(1+$F$23/100)/(($A$28-$F$23)/100),DCF_Base!$L$19*DCF_Base!$B$29),DCF_Base!$L$19*DCF_Base!$B$29))/(1+$A$28/100)^DCF_Base!$L$4+Assumptions!$B$5-Assumptions!$B$4)/Assumptions!$B$3*Assumptions!$B$10</f>
-        <v>175.921217924232</v>
+        <v>190.259361666075</v>
       </c>
     </row>
   </sheetData>

</xml_diff>